<commit_message>
Recover Total Hours grand total when source BB9 is #VALUE!
When a time cell (Start/Stop/Lunch) contains non-time text like "OFF",
the per-day Total Hours formula returns #VALUE! and the weekly grand
total BB9 =SUM(L9:BA9) propagates that error. Fall back to summing the
valid daily Total Hours we already extracted, so the TOTALS row carries
a real number and the QA_Flag explains the substitution.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/extracted.xlsx
+++ b/output/extracted.xlsx
@@ -1236,6 +1236,9 @@
           <t>TOTALS</t>
         </is>
       </c>
+      <c r="O9" t="n">
+        <v>94</v>
+      </c>
       <c r="P9" t="n">
         <v>32</v>
       </c>
@@ -1256,7 +1259,7 @@
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>TOTALS; grand_total_hours='#VALUE!'</t>
+          <t>TOTALS; Total Hours computed (BB9='#VALUE!')</t>
         </is>
       </c>
     </row>
@@ -2566,6 +2569,9 @@
           <t>TOTALS</t>
         </is>
       </c>
+      <c r="O25" t="n">
+        <v>95</v>
+      </c>
       <c r="P25" t="n">
         <v>32</v>
       </c>
@@ -2586,7 +2592,7 @@
       </c>
       <c r="X25" s="2" t="inlineStr">
         <is>
-          <t>TOTALS; grand_total_hours='#VALUE!'</t>
+          <t>TOTALS; Total Hours computed (BB9='#VALUE!')</t>
         </is>
       </c>
     </row>
@@ -7483,8 +7489,8 @@
       <c r="W2" t="n">
         <v>94</v>
       </c>
-      <c r="X2" t="e">
-        <v>#VALUE!</v>
+      <c r="X2" t="n">
+        <v>94</v>
       </c>
       <c r="Y2" s="7" t="inlineStr">
         <is>
@@ -7687,8 +7693,8 @@
       <c r="W4" t="n">
         <v>95</v>
       </c>
-      <c r="X4" t="e">
-        <v>#VALUE!</v>
+      <c r="X4" t="n">
+        <v>95</v>
       </c>
       <c r="Y4" s="7" t="inlineStr">
         <is>
@@ -8499,7 +8505,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-21 02:22:54</t>
+          <t>2026-05-21 15:57:28</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>

<commit_message>
Improve QA_Flag wording and add diagnostic probe scripts
- QA_Flag now reports the exact bad cell address and contents
  (e.g. "Start cell L5 = 'OFF' — not a time") instead of the generic
  "total_hrs='#VALUE!'". Detection is structural — anything in a time
  cell that isn't a datetime/time/float-fraction-of-day is flagged.
- Drop the "TOTALS" literal from QA_Flag; clean TOTALS rows now read
  "OK" too. Grey tint for TOTALS rows is driven off the Day column
  instead of the flag string.
- Add scripts/probe_value_errors.py and scripts/show_current_output.py
  for ad-hoc inspection during diagnosis.
- Include output/extracted_v2.xlsx and extracted_v3.xlsx as historical
  snapshots of intermediate flag-wording iterations.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/extracted.xlsx
+++ b/output/extracted.xlsx
@@ -672,7 +672,7 @@
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>total_hrs='#VALUE!'</t>
+          <t>Start cell L5 = 'OFF' — not a time</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>TOTALS; Total Hours computed (BB9='#VALUE!')</t>
+          <t>Total Hours cell BB9 = '#VALUE!' — recomputed from day rows</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="X17" s="4" t="inlineStr">
         <is>
-          <t>TOTALS</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="X18" s="2" t="inlineStr">
         <is>
-          <t>total_hrs='#VALUE!'</t>
+          <t>Start cell L5 = 'OFF' — not a time</t>
         </is>
       </c>
     </row>
@@ -2592,7 +2592,7 @@
       </c>
       <c r="X25" s="2" t="inlineStr">
         <is>
-          <t>TOTALS; Total Hours computed (BB9='#VALUE!')</t>
+          <t>Total Hours cell BB9 = '#VALUE!' — recomputed from day rows</t>
         </is>
       </c>
     </row>
@@ -3265,7 +3265,7 @@
       </c>
       <c r="X33" s="4" t="inlineStr">
         <is>
-          <t>TOTALS</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -3938,7 +3938,7 @@
       </c>
       <c r="X41" s="4" t="inlineStr">
         <is>
-          <t>TOTALS</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -4611,7 +4611,7 @@
       </c>
       <c r="X49" s="4" t="inlineStr">
         <is>
-          <t>TOTALS</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -5284,7 +5284,7 @@
       </c>
       <c r="X57" s="4" t="inlineStr">
         <is>
-          <t>TOTALS</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -5947,7 +5947,7 @@
       </c>
       <c r="X65" s="4" t="inlineStr">
         <is>
-          <t>TOTALS</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -6620,7 +6620,7 @@
       </c>
       <c r="X73" s="4" t="inlineStr">
         <is>
-          <t>TOTALS</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -7223,7 +7223,7 @@
       </c>
       <c r="X81" s="4" t="inlineStr">
         <is>
-          <t>TOTALS</t>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -8505,7 +8505,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-05-21 15:57:28</t>
+          <t>2026-05-21 15:58:13</t>
         </is>
       </c>
       <c r="E2" t="n">

</xml_diff>